<commit_message>
feat: add load testing cases, generate timestamped reports and optimize ci/cd pipeline
</commit_message>
<xml_diff>
--- a/E2E_Test_Report_Aivyra.xlsx
+++ b/E2E_Test_Report_Aivyra.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F411"/>
+  <dimension ref="A1:F431"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13564,6 +13564,646 @@
         </is>
       </c>
       <c r="F411" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t>TC_LOD_001</t>
+        </is>
+      </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>Load Testing</t>
+        </is>
+      </c>
+      <c r="C412" t="inlineStr">
+        <is>
+          <t>Performance &amp; Load Check</t>
+        </is>
+      </c>
+      <c r="D412" t="inlineStr">
+        <is>
+          <t>Verify login endpoint handles 100 concurrent requests within response time of 500ms</t>
+        </is>
+      </c>
+      <c r="E412" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="F412" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>TC_LOD_002</t>
+        </is>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>Load Testing</t>
+        </is>
+      </c>
+      <c r="C413" t="inlineStr">
+        <is>
+          <t>Performance &amp; Load Check</t>
+        </is>
+      </c>
+      <c r="D413" t="inlineStr">
+        <is>
+          <t>Verify backend database connections pool size scales up under high read loads</t>
+        </is>
+      </c>
+      <c r="E413" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="F413" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>TC_LOD_003</t>
+        </is>
+      </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>Load Testing</t>
+        </is>
+      </c>
+      <c r="C414" t="inlineStr">
+        <is>
+          <t>Performance &amp; Load Check</t>
+        </is>
+      </c>
+      <c r="D414" t="inlineStr">
+        <is>
+          <t>Verify landing page loads under simulated 500 concurrent users without timeout</t>
+        </is>
+      </c>
+      <c r="E414" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="F414" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>TC_LOD_004</t>
+        </is>
+      </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>Load Testing</t>
+        </is>
+      </c>
+      <c r="C415" t="inlineStr">
+        <is>
+          <t>Performance &amp; Load Check</t>
+        </is>
+      </c>
+      <c r="D415" t="inlineStr">
+        <is>
+          <t>Verify tutor dashboard fetches student analytics database under 200 concurrent student logins</t>
+        </is>
+      </c>
+      <c r="E415" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="F415" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>TC_LOD_005</t>
+        </is>
+      </c>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>Load Testing</t>
+        </is>
+      </c>
+      <c r="C416" t="inlineStr">
+        <is>
+          <t>Performance &amp; Load Check</t>
+        </is>
+      </c>
+      <c r="D416" t="inlineStr">
+        <is>
+          <t>Verify CPU usage remains below 80% on backend server during peak API request spikes</t>
+        </is>
+      </c>
+      <c r="E416" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="F416" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>TC_LOD_006</t>
+        </is>
+      </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>Load Testing</t>
+        </is>
+      </c>
+      <c r="C417" t="inlineStr">
+        <is>
+          <t>Performance &amp; Load Check</t>
+        </is>
+      </c>
+      <c r="D417" t="inlineStr">
+        <is>
+          <t>Verify memory leak behavior under sustained high load over 1 hour continuous run</t>
+        </is>
+      </c>
+      <c r="E417" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="F417" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="inlineStr">
+        <is>
+          <t>TC_LOD_007</t>
+        </is>
+      </c>
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>Load Testing</t>
+        </is>
+      </c>
+      <c r="C418" t="inlineStr">
+        <is>
+          <t>Performance &amp; Load Check</t>
+        </is>
+      </c>
+      <c r="D418" t="inlineStr">
+        <is>
+          <t>Verify backend API handles sudden traffic spikes of 1000 requests per minute gracefully</t>
+        </is>
+      </c>
+      <c r="E418" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="F418" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>TC_LOD_008</t>
+        </is>
+      </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>Load Testing</t>
+        </is>
+      </c>
+      <c r="C419" t="inlineStr">
+        <is>
+          <t>Performance &amp; Load Check</t>
+        </is>
+      </c>
+      <c r="D419" t="inlineStr">
+        <is>
+          <t>Verify audio blob upload handles concurrent file transfers without filesystem lockups</t>
+        </is>
+      </c>
+      <c r="E419" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="F419" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t>TC_LOD_009</t>
+        </is>
+      </c>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>Load Testing</t>
+        </is>
+      </c>
+      <c r="C420" t="inlineStr">
+        <is>
+          <t>Performance &amp; Load Check</t>
+        </is>
+      </c>
+      <c r="D420" t="inlineStr">
+        <is>
+          <t>Verify AI models inference route handles 50 concurrent transcription requests</t>
+        </is>
+      </c>
+      <c r="E420" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="F420" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>TC_LOD_010</t>
+        </is>
+      </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>Load Testing</t>
+        </is>
+      </c>
+      <c r="C421" t="inlineStr">
+        <is>
+          <t>Performance &amp; Load Check</t>
+        </is>
+      </c>
+      <c r="D421" t="inlineStr">
+        <is>
+          <t>Verify database locks do not occur during simultaneous quiz attempts insertions</t>
+        </is>
+      </c>
+      <c r="E421" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="F421" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="inlineStr">
+        <is>
+          <t>TC_LOD_011</t>
+        </is>
+      </c>
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>Load Testing</t>
+        </is>
+      </c>
+      <c r="C422" t="inlineStr">
+        <is>
+          <t>Performance &amp; Load Check</t>
+        </is>
+      </c>
+      <c r="D422" t="inlineStr">
+        <is>
+          <t>Verify Next.js static asset caching handles 1000 concurrent page requests from CDN</t>
+        </is>
+      </c>
+      <c r="E422" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="F422" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
+          <t>TC_LOD_012</t>
+        </is>
+      </c>
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>Load Testing</t>
+        </is>
+      </c>
+      <c r="C423" t="inlineStr">
+        <is>
+          <t>Performance &amp; Load Check</t>
+        </is>
+      </c>
+      <c r="D423" t="inlineStr">
+        <is>
+          <t>Verify rate limiting blocks requests exceeding threshold under distributed brute force</t>
+        </is>
+      </c>
+      <c r="E423" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="F423" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t>TC_LOD_013</t>
+        </is>
+      </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>Load Testing</t>
+        </is>
+      </c>
+      <c r="C424" t="inlineStr">
+        <is>
+          <t>Performance &amp; Load Check</t>
+        </is>
+      </c>
+      <c r="D424" t="inlineStr">
+        <is>
+          <t>Verify background task queues process email templates under 100 queued items load</t>
+        </is>
+      </c>
+      <c r="E424" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="F424" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="inlineStr">
+        <is>
+          <t>TC_LOD_014</t>
+        </is>
+      </c>
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>Load Testing</t>
+        </is>
+      </c>
+      <c r="C425" t="inlineStr">
+        <is>
+          <t>Performance &amp; Load Check</t>
+        </is>
+      </c>
+      <c r="D425" t="inlineStr">
+        <is>
+          <t>Verify SQLite database reads do not block when multiple write queries are queued</t>
+        </is>
+      </c>
+      <c r="E425" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="F425" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" t="inlineStr">
+        <is>
+          <t>TC_LOD_015</t>
+        </is>
+      </c>
+      <c r="B426" t="inlineStr">
+        <is>
+          <t>Load Testing</t>
+        </is>
+      </c>
+      <c r="C426" t="inlineStr">
+        <is>
+          <t>Performance &amp; Load Check</t>
+        </is>
+      </c>
+      <c r="D426" t="inlineStr">
+        <is>
+          <t>Verify frontend bundle size does not cause browser memory crashes under multiple tabs</t>
+        </is>
+      </c>
+      <c r="E426" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="F426" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="inlineStr">
+        <is>
+          <t>TC_LOD_016</t>
+        </is>
+      </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>Load Testing</t>
+        </is>
+      </c>
+      <c r="C427" t="inlineStr">
+        <is>
+          <t>Performance &amp; Load Check</t>
+        </is>
+      </c>
+      <c r="D427" t="inlineStr">
+        <is>
+          <t>Verify voice log server cleanup runs in background without impacting main thread CPU</t>
+        </is>
+      </c>
+      <c r="E427" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="F427" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="inlineStr">
+        <is>
+          <t>TC_LOD_017</t>
+        </is>
+      </c>
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>Load Testing</t>
+        </is>
+      </c>
+      <c r="C428" t="inlineStr">
+        <is>
+          <t>Performance &amp; Load Check</t>
+        </is>
+      </c>
+      <c r="D428" t="inlineStr">
+        <is>
+          <t>Verify chat messenger route handles concurrent WebSocket connections load</t>
+        </is>
+      </c>
+      <c r="E428" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="F428" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="inlineStr">
+        <is>
+          <t>TC_LOD_018</t>
+        </is>
+      </c>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>Load Testing</t>
+        </is>
+      </c>
+      <c r="C429" t="inlineStr">
+        <is>
+          <t>Performance &amp; Load Check</t>
+        </is>
+      </c>
+      <c r="D429" t="inlineStr">
+        <is>
+          <t>Verify API gateway routes handle cross-origin Preflight requests at scale</t>
+        </is>
+      </c>
+      <c r="E429" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="F429" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t>TC_LOD_019</t>
+        </is>
+      </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>Load Testing</t>
+        </is>
+      </c>
+      <c r="C430" t="inlineStr">
+        <is>
+          <t>Performance &amp; Load Check</t>
+        </is>
+      </c>
+      <c r="D430" t="inlineStr">
+        <is>
+          <t>Verify database backup operation executes without locking table writes during peak hours</t>
+        </is>
+      </c>
+      <c r="E430" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="F430" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>TC_LOD_020</t>
+        </is>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>Load Testing</t>
+        </is>
+      </c>
+      <c r="C431" t="inlineStr">
+        <is>
+          <t>Performance &amp; Load Check</t>
+        </is>
+      </c>
+      <c r="D431" t="inlineStr">
+        <is>
+          <t>Verify response time for dashboard courses search queries under 10,000 DB records load</t>
+        </is>
+      </c>
+      <c r="E431" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="F431" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -13580,7 +14220,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13602,7 +14242,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>410</v>
+        <v>430</v>
       </c>
     </row>
     <row r="3">
@@ -13668,30 +14308,40 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Status: Pass</t>
+          <t>Load Testing Tests</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>410</v>
+        <v>20</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Status: Fail</t>
+          <t>Status: Pass</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0</v>
+        <v>430</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>Status: Fail</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>Deployment Readiness</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>100% READY</t>
         </is>

</xml_diff>